<commit_message>
Add gitignore rule, update Excel workbook and cleaning notebook
</commit_message>
<xml_diff>
--- a/data/processed/Excel/insurance_billing_reconciliation.xlsx
+++ b/data/processed/Excel/insurance_billing_reconciliation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ayman\OneDrive\Documents\GitHub\medical_insurance_cost_prediction\data\processed\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{6D77D576-7407-4C8D-853C-BBE68DA65154}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{070A6DDB-0B63-4723-A035-5659D4BE718A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="25500" yWindow="0" windowWidth="25800" windowHeight="20985" xr2:uid="{89D594AC-F36D-4D16-9EEE-174E32618C14}"/>
   </bookViews>
@@ -18498,7 +18498,7 @@
     <col min="1" max="1" width="18.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.28515625" customWidth="1"/>
+    <col min="4" max="4" width="15.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>